<commit_message>
Remove Oat Bathing Bar SKU from listing sheet
That SKU had no images in the source set, so its row could not meet the
sheet's mandatory Image-1/Image-2 requirement. All 9 remaining rows carry
three image links each.

The deleted row's formula (U13) went with it; every other formula is a
same-row reference and none pointed at row 13, so no references needed
fixing. Recalc reports 0 errors across the remaining 13 formulas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013FiyhpU9srtNh8Sg6p6Gc3
</commit_message>
<xml_diff>
--- a/OTC_Listing_Format_-_Tuco_Kids_10_SKUs_v3_with_image_links.xlsx
+++ b/OTC_Listing_Format_-_Tuco_Kids_10_SKUs_v3_with_image_links.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="230">
   <si>
     <t xml:space="preserve">Mandatory</t>
   </si>
@@ -736,33 +736,6 @@
   </si>
   <si>
     <t xml:space="preserve">For external use only. Avoid applying near eyes, mouth, or on cuts and broken skin. Do not apply on children's hands as they may touch their eyes or mouth. Use under adult supervision. Discontinue if irritation occurs. Store in a cool, dry place.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">65055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tuco Kids Oat Bathing Bar 75g (Pack of 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anuspa Heritage Private Limited</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8906191251578</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oat Extract, Allantoin, Rice Water, Licorice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tuco Kids Oat Bathing Bar is a gentle, soap-free, pH 5.5 bathing bar specially crafted for babies and kids with delicate or sensitive skin. Enriched with Oat Extract, Allantoin, Rice Water and Licorice, it soothes irritation, locks in moisture and strengthens the skin barrier. Dermatologically tested and suitable for skin prone to dryness, eczema or allergies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oat Extract - soothes and protects dry, sensitive skin; Allantoin - calms irritation; Rice Water - nourishes and softens; Licorice - soothes and evens skin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soap-free, pH 5.5 balanced; Ultra-mild for babies and sensitive skin; Locks in moisture; Strengthens skin barrier; Dermatologically tested</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Can be used on face and body. Lather into wet skin and rinse clean with water.</t>
   </si>
 </sst>
 </file>
@@ -3124,156 +3097,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>231</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="G13" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" s="23" t="s">
-        <v>232</v>
-      </c>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="K13" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="L13" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="M13" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="N13" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="O13" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="P13" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q13" s="24" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="R13" s="23" t="n">
-        <v>220</v>
-      </c>
-      <c r="S13" s="23" t="n">
-        <v>179</v>
-      </c>
-      <c r="T13" s="23"/>
-      <c r="U13" s="25" t="n">
-        <f aca="false">R13*(1-32%)</f>
-        <v>149.6</v>
-      </c>
-      <c r="V13" s="23"/>
-      <c r="W13" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="X13" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y13" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="Z13" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA13" s="23" t="n">
-        <v>75</v>
-      </c>
-      <c r="AB13" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="AC13" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="AD13" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="AE13" s="23" t="s">
-        <v>234</v>
-      </c>
-      <c r="AF13" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="AG13" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH13" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="AI13" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="AJ13" s="23" t="n">
-        <v>75</v>
-      </c>
-      <c r="AK13" s="23" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="AL13" s="23" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="AM13" s="23" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="AN13" s="23"/>
-      <c r="AO13" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="AP13" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="AQ13" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="AR13" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="AS13" s="23"/>
-      <c r="AT13" s="23"/>
-      <c r="AU13" s="23"/>
-      <c r="AV13" s="23"/>
-      <c r="AW13" s="23"/>
-      <c r="AX13" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="AY13" s="23" t="s">
-        <v>236</v>
-      </c>
-      <c r="AZ13" s="23" t="s">
-        <v>237</v>
-      </c>
-      <c r="BA13" s="23" t="s">
-        <v>238</v>
-      </c>
-      <c r="BB13" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="BC13" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="BD13" s="23" t="s">
-        <v>89</v>
-      </c>
-    </row>
+    <row r="13" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C1:T1"/>

</xml_diff>

<commit_message>
Make image links clickable in listing sheet
The 27 Drive URLs in Image-1/2/3 were plain text. Each cell now carries a
real hyperlink target alongside its display text, styled blue and
underlined so it reads as a link.

Verified the links survive the LibreOffice recalc rewrite: all 27 cells
load back with a hyperlink target matching their text.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013FiyhpU9srtNh8Sg6p6Gc3
</commit_message>
<xml_diff>
--- a/OTC_Listing_Format_-_Tuco_Kids_10_SKUs_v3_with_image_links.xlsx
+++ b/OTC_Listing_Format_-_Tuco_Kids_10_SKUs_v3_with_image_links.xlsx
@@ -748,7 +748,7 @@
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -804,6 +804,14 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -935,7 +943,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1041,6 +1049,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1796,13 +1808,13 @@
       <c r="AR4" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS4" s="23" t="s">
+      <c r="AS4" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="AT4" s="23" t="s">
+      <c r="AT4" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="AU4" s="23" t="s">
+      <c r="AU4" s="27" t="s">
         <v>107</v>
       </c>
       <c r="AV4" s="23"/>
@@ -1954,13 +1966,13 @@
       <c r="AR5" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS5" s="23" t="s">
+      <c r="AS5" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="AT5" s="23" t="s">
+      <c r="AT5" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="AU5" s="23" t="s">
+      <c r="AU5" s="27" t="s">
         <v>122</v>
       </c>
       <c r="AV5" s="23"/>
@@ -2113,13 +2125,13 @@
       <c r="AR6" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS6" s="23" t="s">
+      <c r="AS6" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AT6" s="23" t="s">
+      <c r="AT6" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="AU6" s="23" t="s">
+      <c r="AU6" s="27" t="s">
         <v>139</v>
       </c>
       <c r="AV6" s="23"/>
@@ -2272,13 +2284,13 @@
       <c r="AR7" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS7" s="23" t="s">
+      <c r="AS7" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="AT7" s="23" t="s">
+      <c r="AT7" s="27" t="s">
         <v>154</v>
       </c>
-      <c r="AU7" s="23" t="s">
+      <c r="AU7" s="27" t="s">
         <v>155</v>
       </c>
       <c r="AV7" s="23"/>
@@ -2430,13 +2442,13 @@
       <c r="AR8" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS8" s="23" t="s">
+      <c r="AS8" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="AT8" s="23" t="s">
+      <c r="AT8" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="AU8" s="23" t="s">
+      <c r="AU8" s="27" t="s">
         <v>169</v>
       </c>
       <c r="AV8" s="23"/>
@@ -2589,13 +2601,13 @@
       <c r="AR9" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS9" s="23" t="s">
+      <c r="AS9" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="AT9" s="23" t="s">
+      <c r="AT9" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="AU9" s="23" t="s">
+      <c r="AU9" s="27" t="s">
         <v>182</v>
       </c>
       <c r="AV9" s="23"/>
@@ -2747,13 +2759,13 @@
       <c r="AR10" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS10" s="23" t="s">
+      <c r="AS10" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="AT10" s="23" t="s">
+      <c r="AT10" s="27" t="s">
         <v>193</v>
       </c>
-      <c r="AU10" s="23" t="s">
+      <c r="AU10" s="27" t="s">
         <v>194</v>
       </c>
       <c r="AV10" s="23"/>
@@ -2906,13 +2918,13 @@
       <c r="AR11" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS11" s="23" t="s">
+      <c r="AS11" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="AT11" s="23" t="s">
+      <c r="AT11" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="AU11" s="23" t="s">
+      <c r="AU11" s="27" t="s">
         <v>210</v>
       </c>
       <c r="AV11" s="23"/>
@@ -3064,13 +3076,13 @@
       <c r="AR12" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AS12" s="23" t="s">
+      <c r="AS12" s="27" t="s">
         <v>222</v>
       </c>
-      <c r="AT12" s="23" t="s">
+      <c r="AT12" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="AU12" s="23" t="s">
+      <c r="AU12" s="27" t="s">
         <v>224</v>
       </c>
       <c r="AV12" s="23"/>
@@ -3105,6 +3117,35 @@
     <mergeCell ref="AO1:AR1"/>
     <mergeCell ref="AX1:BD1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="AS4" r:id="rId1" display="https://drive.google.com/file/d/1ojWdYnCJPWy2Xry-GwUgrazq6poDKA46/view?usp=sharing"/>
+    <hyperlink ref="AT4" r:id="rId2" display="https://drive.google.com/file/d/1MDYo51NrfGPkuBgTsGfLFFiV2VMNFJL-/view?usp=sharing"/>
+    <hyperlink ref="AU4" r:id="rId3" display="https://drive.google.com/file/d/1S0NjAbs1t2PnUT5WwkgoCC0DZEd7LZkj/view?usp=sharing"/>
+    <hyperlink ref="AS5" r:id="rId4" display="https://drive.google.com/file/d/1hjMuxQFD3OMfm1LAD-V9o5ORxUsBJaf3/view?usp=sharing"/>
+    <hyperlink ref="AT5" r:id="rId5" display="https://drive.google.com/file/d/1TnwNh-Ns5sfxEvVs9yuNhuzc81QPA1w5/view?usp=sharing"/>
+    <hyperlink ref="AU5" r:id="rId6" display="https://drive.google.com/file/d/1yuGNdOGkSV1Ue9oAf1j-b1rGPck6FXjM/view?usp=sharing"/>
+    <hyperlink ref="AS6" r:id="rId7" display="https://drive.google.com/file/d/1UdZHk7EgjZvW_xLjQIhK8M6aPiFte948/view?usp=sharing"/>
+    <hyperlink ref="AT6" r:id="rId8" display="https://drive.google.com/file/d/14hvZZGQhXwXwRrOJJdKCLJE3medAwp9Q/view?usp=sharing"/>
+    <hyperlink ref="AU6" r:id="rId9" display="https://drive.google.com/file/d/10rPjU5WyUX4xxGCrZ5h_yqB_zt8JCHxS/view?usp=sharing"/>
+    <hyperlink ref="AS7" r:id="rId10" display="https://drive.google.com/file/d/1umHrvjv06YnpqEHCoWrbCxMw4MTp6JzN/view?usp=sharing"/>
+    <hyperlink ref="AT7" r:id="rId11" display="https://drive.google.com/file/d/1i1mF2QO-_Vq26uORz9_jA3_I2tlEKnhk/view?usp=sharing"/>
+    <hyperlink ref="AU7" r:id="rId12" display="https://drive.google.com/file/d/1NH_1N1TkxW9ACirUh1FoaU31rp2DxRXN/view?usp=sharing"/>
+    <hyperlink ref="AS8" r:id="rId13" display="https://drive.google.com/file/d/1zAMS6K6sWCh_NqpWCm7SdjZNAMQ2uKtR/view?usp=sharing"/>
+    <hyperlink ref="AT8" r:id="rId14" display="https://drive.google.com/file/d/1fmFzwud8FrECv-RwU9OfIZuVjcbvNmmj/view?usp=sharing"/>
+    <hyperlink ref="AU8" r:id="rId15" display="https://drive.google.com/file/d/1FR3-uayY0T8GsnBWnZIYNRBbWr2clFur/view?usp=sharing"/>
+    <hyperlink ref="AS9" r:id="rId16" display="https://drive.google.com/file/d/1cTQRotWPDhHA_RtCwpVskOSR-sMYpr8K/view?usp=sharing"/>
+    <hyperlink ref="AT9" r:id="rId17" display="https://drive.google.com/file/d/1rXHQPKDfXCNRms8f1pN1lp0gGPi8A_-f/view?usp=sharing"/>
+    <hyperlink ref="AU9" r:id="rId18" display="https://drive.google.com/file/d/16YmfYP-0aJSy9OVJtyX-LoFR-6UuPD_y/view?usp=sharing"/>
+    <hyperlink ref="AS10" r:id="rId19" display="https://drive.google.com/file/d/18wk--a6LK37uWyiUke-j8VBr8GPyXe9p/view?usp=sharing"/>
+    <hyperlink ref="AT10" r:id="rId20" display="https://drive.google.com/file/d/1TYR8F2kH5989Ig2XyV-VJV7UWFag3b4W/view?usp=sharing"/>
+    <hyperlink ref="AU10" r:id="rId21" display="https://drive.google.com/file/d/1We8eX5a5-Ookx9D6GWYnZqb3-GDq9oTQ/view?usp=sharing"/>
+    <hyperlink ref="AS11" r:id="rId22" display="https://drive.google.com/file/d/1hUNAArHtCA4s-z369ryqC0Vus224hnjC/view?usp=sharing"/>
+    <hyperlink ref="AT11" r:id="rId23" display="https://drive.google.com/file/d/1MbocXL41HpC-Y-OXbX9pw4Odbk34tyIb/view?usp=sharing"/>
+    <hyperlink ref="AU11" r:id="rId24" display="https://drive.google.com/file/d/1hIKX0vLKsZw5VYjm_Eq6gKU38G4PwXq7/view?usp=sharing"/>
+    <hyperlink ref="AS12" r:id="rId25" display="https://drive.google.com/file/d/14xwU3kZ_G1qqrzXsCocsRew3Pr2ogTmE/view?usp=sharing"/>
+    <hyperlink ref="AT12" r:id="rId26" display="https://drive.google.com/file/d/1hOabuPnhlME44_vUeBXzDIjcRipyS1b0/view?usp=sharing"/>
+    <hyperlink ref="AU12" r:id="rId27" display="https://drive.google.com/file/d/11kC1g7ONIDJLAFmnj-hIU9_AMVgZJJq_/view?usp=sharing"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Use per-product folder links instead of individual image links
Replaces the three per-image Drive links with a single clickable link to
that product's folder, matching the sheet's own guidance under the image
columns ("Share separate folder links for each SKU/product").

The folder link goes in AS (Image-1); AT and AU are cleared rather than
repeating the same URL three times. All 9 links are distinct and point at
the folder for their row's product.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013FiyhpU9srtNh8Sg6p6Gc3
</commit_message>
<xml_diff>
--- a/OTC_Listing_Format_-_Tuco_Kids_10_SKUs_v3_with_image_links.xlsx
+++ b/OTC_Listing_Format_-_Tuco_Kids_10_SKUs_v3_with_image_links.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="212">
   <si>
     <t xml:space="preserve">Mandatory</t>
   </si>
@@ -363,13 +363,7 @@
     <t xml:space="preserve">Child</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1ojWdYnCJPWy2Xry-GwUgrazq6poDKA46/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1MDYo51NrfGPkuBgTsGfLFFiV2VMNFJL-/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1S0NjAbs1t2PnUT5WwkgoCC0DZEd7LZkj/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1yP0mxPJhdgPbR_s79_MmLFm8sYI0-gdb?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids 2-in-1 Face Cream + Sunscreen SPF 50 is a daily face cream and sunscreen in one, made for kids aged 2-15. It shields delicate skin from harmful UVA/UVB rays with broad-spectrum PA++++ protection while moisturising and evening out skin tone. The lightweight, non-greasy formula leaves no white cast and does not feel sticky or heavy on young faces.</t>
@@ -408,13 +402,7 @@
     <t xml:space="preserve">Aloe Vera</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1hjMuxQFD3OMfm1LAD-V9o5ORxUsBJaf3/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1TnwNh-Ns5sfxEvVs9yuNhuzc81QPA1w5/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1yuGNdOGkSV1Ue9oAf1j-b1rGPck6FXjM/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1jFOX8x5PyO-MDKmMh9RHKWpgABZ-T2jI?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Gel Sunscreen SPF 50 is a lightweight, fast-absorbing gel sunscreen for kids aged 2-15 that provides broad-spectrum UVA/UVB protection with PA++++. Enriched with soothing Aloe Vera, it calms and hydrates skin while helping prevent sunburn, tanning and long-term sun damage. Benzophenone-3 and Avobenzone free, non-greasy and ideal for daily wear at school, playtime and outdoors.</t>
@@ -459,13 +447,7 @@
     <t xml:space="preserve">Skin Care</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1UdZHk7EgjZvW_xLjQIhK8M6aPiFte948/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/14hvZZGQhXwXwRrOJJdKCLJE3medAwp9Q/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/10rPjU5WyUX4xxGCrZ5h_yqB_zt8JCHxS/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1AXhoTNn1WFYVBmDmYVGPnRJLoNuc1GcK?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Kumkumadi Body Lotion is an Ayurvedic body lotion for kids aged 3-12, crafted with Kumkumadi, Haldi, Manjistha and Red Sandalwood to nourish skin and support its natural glow. Squalane, Rose Water and Vitamin E add lightweight, non-greasy moisture and antioxidant care. Dermatologically and clinically tested, and free from sulphates and parabens.</t>
@@ -507,13 +489,7 @@
     <t xml:space="preserve">Skin Care / Bath</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1umHrvjv06YnpqEHCoWrbCxMw4MTp6JzN/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1i1mF2QO-_Vq26uORz9_jA3_I2tlEKnhk/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1NH_1N1TkxW9ACirUh1FoaU31rp2DxRXN/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1Kn3zQ2TjI-Z_pSl68ySUC-9QEAPxW7MU?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Kumkumadi Soap is a dermatologically tested Ayurvedic bathing bar for kids aged 3-12, made with Kumkumadi, Manjistha, Red Sandalwood and Haldi. It gently cleanses while nourishing skin and supporting its natural radiance, without stripping moisture. 90%+ natural origin and free from parabens, SLS and phthalates. Pack of 2 bars, 75g each.</t>
@@ -549,13 +525,7 @@
     <t xml:space="preserve">Kakadu Plum, Orange, Green Tea, Yogurt</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1zAMS6K6sWCh_NqpWCm7SdjZNAMQ2uKtR/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1fmFzwud8FrECv-RwU9OfIZuVjcbvNmmj/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1FR3-uayY0T8GsnBWnZIYNRBbWr2clFur/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1--OQ7u1bta3auUdssAOvANlM_OuQiwSh?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Bye Dull Skin Body Wash is a gentle brightening body wash for active kids, made to refresh dull-looking skin after school, sports and outdoor play. Kakadu Plum, Orange, Green Tea and Yogurt wash away dirt, dust and pollution while supporting a healthy natural glow. Dermatologically tested and free from SLS, parabens, phthalates and skin lighteners.</t>
@@ -588,13 +558,7 @@
     <t xml:space="preserve">Orange, Witch Hazel, Glycerin, Sugarcane</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1cTQRotWPDhHA_RtCwpVskOSR-sMYpr8K/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1rXHQPKDfXCNRms8f1pN1lp0gGPi8A_-f/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/16YmfYP-0aJSy9OVJtyX-LoFR-6UuPD_y/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1c0mnshaI1ujk8pprI4qJ7qiXcjMrVSHs?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Daily Face Wash is a gentle, pH-balanced gel face wash made for kids with oily or acne-prone skin. Enriched with Orange, Witch Hazel, Glycerin and Sugarcane, it helps balance excess oil, cleanse pores and keep skin clear and fresh. Dermatologically tested and free from parabens, SLS and sulphates; suitable for kids aged 2-15.</t>
@@ -624,13 +588,7 @@
     <t xml:space="preserve">Skin Care / Hair Care / Bath</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/18wk--a6LK37uWyiUke-j8VBr8GPyXe9p/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1TYR8F2kH5989Ig2XyV-VJV7UWFag3b4W/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1We8eX5a5-Ookx9D6GWYnZqb3-GDq9oTQ/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1W2AU9JUfyl_QFj6OUIehl_ix4VNvqI-W?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids 3-in-1 Head to Toe Wash is one gentle formula that cleanses hair, face and body, replacing separate shampoo, body wash and face wash for kids aged 3-12. Oat Extract soothes, Rice Water strengthens hair, Almond Oil nourishes and Green Gram Extract cleanses without stripping natural oils. Tear-free, pH-balanced, 97% natural origin and free from parabens, SLS and phthalates.</t>
@@ -672,13 +630,7 @@
     <t xml:space="preserve">Hand Hygiene</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1hUNAArHtCA4s-z369ryqC0Vus224hnjC/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1MbocXL41HpC-Y-OXbX9pw4Odbk34tyIb/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1hIKX0vLKsZw5VYjm_Eq6gKU38G4PwXq7/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1k3T5Ys14H5-t8kIDUY1nKzM9oEpxfpYV?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Alcohol-Free Hand Sanitiser gives kids effective germ protection without the dryness and sting of alcohol-based sanitisers. Made with Tulsi, Neem and Clove, it cleans hands on the go while keeping little hands soft and nourished. No water needed; SLS and paraben free, suitable for kids aged 3+.</t>
@@ -714,13 +666,7 @@
     <t xml:space="preserve">Skin Care / Mosquito Repellent</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/14xwU3kZ_G1qqrzXsCocsRew3Pr2ogTmE/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/1hOabuPnhlME44_vUeBXzDIjcRipyS1b0/view?usp=sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/file/d/11kC1g7ONIDJLAFmnj-hIU9_AMVgZJJq_/view?usp=sharing</t>
+    <t xml:space="preserve">https://drive.google.com/drive/folders/1EFJ1SJS3AjAbHOzTtWMO0-ieMek5WyxN?usp=sharing</t>
   </si>
   <si>
     <t xml:space="preserve">Tuco Kids Don't Bug Me Mosquito Repellent Lotion is a DEET-free 2-in-1 lotion that protects kids from mosquito bites for up to 8 hours while soothing the skin. Aloe Vera, Chamomile and Calendula oils calm itchy skin and keep it moisturised. Lightweight and non-sticky with a mild scent, free from SLS, parabens and phthalates, in a mess-free travel tube.</t>
@@ -1811,28 +1757,24 @@
       <c r="AS4" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="AT4" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="AU4" s="27" t="s">
-        <v>107</v>
-      </c>
+      <c r="AT4" s="23"/>
+      <c r="AU4" s="23"/>
       <c r="AV4" s="23"/>
       <c r="AW4" s="23"/>
       <c r="AX4" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="AY4" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="AZ4" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="AY4" s="23" t="s">
+      <c r="BA4" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="AZ4" s="23" t="s">
+      <c r="BB4" s="23" t="s">
         <v>110</v>
-      </c>
-      <c r="BA4" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="BB4" s="23" t="s">
-        <v>112</v>
       </c>
       <c r="BC4" s="23" t="s">
         <v>89</v>
@@ -1843,10 +1785,10 @@
     </row>
     <row r="5" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="23" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D5" s="23" t="s">
         <v>83</v>
@@ -1861,10 +1803,10 @@
         <v>86</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J5" s="23" t="s">
         <v>89</v>
@@ -1903,13 +1845,13 @@
       </c>
       <c r="V5" s="23"/>
       <c r="W5" s="23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="X5" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y5" s="26" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="Z5" s="23" t="n">
         <v>1</v>
@@ -1927,7 +1869,7 @@
         <v>99</v>
       </c>
       <c r="AE5" s="23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AF5" s="23" t="s">
         <v>101</v>
@@ -1967,30 +1909,26 @@
         <v>102</v>
       </c>
       <c r="AS5" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="AT5" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="AU5" s="27" t="s">
-        <v>122</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="AT5" s="23"/>
+      <c r="AU5" s="23"/>
       <c r="AV5" s="23"/>
       <c r="AW5" s="23"/>
       <c r="AX5" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="AY5" s="23" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="AZ5" s="23" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="BA5" s="23" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="BB5" s="23" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="BC5" s="23" t="s">
         <v>89</v>
@@ -2001,10 +1939,10 @@
     </row>
     <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="23" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D6" s="23" t="s">
         <v>83</v>
@@ -2019,10 +1957,10 @@
         <v>86</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J6" s="23" t="s">
         <v>89</v>
@@ -2040,7 +1978,7 @@
         <v>91</v>
       </c>
       <c r="O6" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="P6" s="23" t="s">
         <v>93</v>
@@ -2062,13 +2000,13 @@
       </c>
       <c r="V6" s="23"/>
       <c r="W6" s="23" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="X6" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y6" s="26" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="Z6" s="23" t="n">
         <v>1</v>
@@ -2077,16 +2015,16 @@
         <v>200</v>
       </c>
       <c r="AB6" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="AC6" s="23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="AD6" s="23" t="s">
         <v>99</v>
       </c>
       <c r="AE6" s="23" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="AF6" s="23" t="s">
         <v>89</v>
@@ -2114,7 +2052,7 @@
       </c>
       <c r="AN6" s="23"/>
       <c r="AO6" s="23" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="AP6" s="23" t="s">
         <v>104</v>
@@ -2126,30 +2064,26 @@
         <v>102</v>
       </c>
       <c r="AS6" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="AT6" s="27" t="s">
-        <v>138</v>
-      </c>
-      <c r="AU6" s="27" t="s">
-        <v>139</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="AT6" s="23"/>
+      <c r="AU6" s="23"/>
       <c r="AV6" s="23"/>
       <c r="AW6" s="23"/>
       <c r="AX6" s="23" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="AY6" s="23" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="AZ6" s="23" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="BA6" s="23" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="BB6" s="23" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="BC6" s="23" t="s">
         <v>89</v>
@@ -2160,10 +2094,10 @@
     </row>
     <row r="7" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="23" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D7" s="23" t="s">
         <v>83</v>
@@ -2178,10 +2112,10 @@
         <v>86</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J7" s="23" t="s">
         <v>89</v>
@@ -2199,10 +2133,10 @@
         <v>91</v>
       </c>
       <c r="O7" s="23" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="P7" s="23" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="Q7" s="24" t="n">
         <v>0.05</v>
@@ -2221,13 +2155,13 @@
       </c>
       <c r="V7" s="23"/>
       <c r="W7" s="23" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="X7" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y7" s="26" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="Z7" s="23" t="n">
         <v>2</v>
@@ -2239,13 +2173,13 @@
         <v>97</v>
       </c>
       <c r="AC7" s="23" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="AD7" s="23" t="s">
         <v>99</v>
       </c>
       <c r="AE7" s="23" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="AF7" s="23" t="s">
         <v>89</v>
@@ -2273,7 +2207,7 @@
       </c>
       <c r="AN7" s="23"/>
       <c r="AO7" s="23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="AP7" s="23" t="s">
         <v>104</v>
@@ -2285,30 +2219,26 @@
         <v>102</v>
       </c>
       <c r="AS7" s="27" t="s">
-        <v>153</v>
-      </c>
-      <c r="AT7" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="AU7" s="27" t="s">
-        <v>155</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="AT7" s="23"/>
+      <c r="AU7" s="23"/>
       <c r="AV7" s="23"/>
       <c r="AW7" s="23"/>
       <c r="AX7" s="23" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="AY7" s="23" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="AZ7" s="23" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="BA7" s="23" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="BB7" s="23" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="BC7" s="23" t="s">
         <v>89</v>
@@ -2319,10 +2249,10 @@
     </row>
     <row r="8" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="23" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>83</v>
@@ -2337,10 +2267,10 @@
         <v>86</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J8" s="23" t="s">
         <v>89</v>
@@ -2358,10 +2288,10 @@
         <v>91</v>
       </c>
       <c r="O8" s="23" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="P8" s="23" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="Q8" s="24" t="n">
         <v>0.18</v>
@@ -2379,13 +2309,13 @@
       </c>
       <c r="V8" s="23"/>
       <c r="W8" s="23" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="X8" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y8" s="26" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="Z8" s="23" t="n">
         <v>1</v>
@@ -2394,16 +2324,16 @@
         <v>200</v>
       </c>
       <c r="AB8" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="AC8" s="23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="AD8" s="23" t="s">
         <v>99</v>
       </c>
       <c r="AE8" s="23" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="AF8" s="23" t="s">
         <v>89</v>
@@ -2431,7 +2361,7 @@
       </c>
       <c r="AN8" s="23"/>
       <c r="AO8" s="23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="AP8" s="23" t="s">
         <v>104</v>
@@ -2443,30 +2373,26 @@
         <v>102</v>
       </c>
       <c r="AS8" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="AT8" s="27" t="s">
-        <v>168</v>
-      </c>
-      <c r="AU8" s="27" t="s">
-        <v>169</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="AT8" s="23"/>
+      <c r="AU8" s="23"/>
       <c r="AV8" s="23"/>
       <c r="AW8" s="23"/>
       <c r="AX8" s="23" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="AY8" s="23" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="AZ8" s="23" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="BA8" s="23" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="BB8" s="23" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="BC8" s="23" t="s">
         <v>89</v>
@@ -2477,10 +2403,10 @@
     </row>
     <row r="9" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="23" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>83</v>
@@ -2516,10 +2442,10 @@
         <v>91</v>
       </c>
       <c r="O9" s="23" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="P9" s="23" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="Q9" s="24" t="n">
         <v>0.18</v>
@@ -2538,13 +2464,13 @@
       </c>
       <c r="V9" s="23"/>
       <c r="W9" s="23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="X9" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y9" s="26" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="Z9" s="23" t="n">
         <v>1</v>
@@ -2553,7 +2479,7 @@
         <v>100</v>
       </c>
       <c r="AB9" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="AC9" s="23" t="s">
         <v>98</v>
@@ -2562,7 +2488,7 @@
         <v>99</v>
       </c>
       <c r="AE9" s="23" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="AF9" s="23" t="s">
         <v>89</v>
@@ -2590,7 +2516,7 @@
       </c>
       <c r="AN9" s="23"/>
       <c r="AO9" s="23" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="AP9" s="23" t="s">
         <v>104</v>
@@ -2602,30 +2528,26 @@
         <v>102</v>
       </c>
       <c r="AS9" s="27" t="s">
-        <v>180</v>
-      </c>
-      <c r="AT9" s="27" t="s">
-        <v>181</v>
-      </c>
-      <c r="AU9" s="27" t="s">
-        <v>182</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="AT9" s="23"/>
+      <c r="AU9" s="23"/>
       <c r="AV9" s="23"/>
       <c r="AW9" s="23"/>
       <c r="AX9" s="23" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="AY9" s="23" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="AZ9" s="23" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="BA9" s="23" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="BB9" s="23" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="BC9" s="23" t="s">
         <v>89</v>
@@ -2636,10 +2558,10 @@
     </row>
     <row r="10" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="23" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D10" s="23" t="s">
         <v>83</v>
@@ -2654,10 +2576,10 @@
         <v>86</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J10" s="23" t="s">
         <v>89</v>
@@ -2675,10 +2597,10 @@
         <v>91</v>
       </c>
       <c r="O10" s="23" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="P10" s="23" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="Q10" s="24" t="n">
         <v>0.18</v>
@@ -2696,13 +2618,13 @@
       </c>
       <c r="V10" s="23"/>
       <c r="W10" s="23" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="X10" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y10" s="23" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="Z10" s="23" t="n">
         <v>1</v>
@@ -2711,16 +2633,16 @@
         <v>300</v>
       </c>
       <c r="AB10" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="AC10" s="23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="AD10" s="23" t="s">
         <v>99</v>
       </c>
       <c r="AE10" s="23" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="AF10" s="23" t="s">
         <v>89</v>
@@ -2748,7 +2670,7 @@
       </c>
       <c r="AN10" s="23"/>
       <c r="AO10" s="23" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="AP10" s="23" t="s">
         <v>104</v>
@@ -2760,30 +2682,26 @@
         <v>102</v>
       </c>
       <c r="AS10" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="AT10" s="27" t="s">
-        <v>193</v>
-      </c>
-      <c r="AU10" s="27" t="s">
-        <v>194</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="AT10" s="23"/>
+      <c r="AU10" s="23"/>
       <c r="AV10" s="23"/>
       <c r="AW10" s="23"/>
       <c r="AX10" s="23" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="AY10" s="23" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="AZ10" s="23" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="BA10" s="23" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="BB10" s="23" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="BC10" s="23" t="s">
         <v>89</v>
@@ -2794,10 +2712,10 @@
     </row>
     <row r="11" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="23" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="D11" s="23" t="s">
         <v>83</v>
@@ -2812,10 +2730,10 @@
         <v>86</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="J11" s="23" t="s">
         <v>89</v>
@@ -2833,10 +2751,10 @@
         <v>91</v>
       </c>
       <c r="O11" s="23" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="P11" s="23" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="Q11" s="24" t="n">
         <v>0.18</v>
@@ -2855,13 +2773,13 @@
       </c>
       <c r="V11" s="23"/>
       <c r="W11" s="23" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="X11" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y11" s="23" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="Z11" s="23" t="n">
         <v>1</v>
@@ -2870,16 +2788,16 @@
         <v>50</v>
       </c>
       <c r="AB11" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="AC11" s="23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="AD11" s="23" t="s">
         <v>99</v>
       </c>
       <c r="AE11" s="23" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="AF11" s="23" t="s">
         <v>89</v>
@@ -2907,7 +2825,7 @@
       </c>
       <c r="AN11" s="23"/>
       <c r="AO11" s="23" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="AP11" s="23" t="s">
         <v>104</v>
@@ -2919,30 +2837,26 @@
         <v>102</v>
       </c>
       <c r="AS11" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="AT11" s="27" t="s">
-        <v>209</v>
-      </c>
-      <c r="AU11" s="27" t="s">
-        <v>210</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="AT11" s="23"/>
+      <c r="AU11" s="23"/>
       <c r="AV11" s="23"/>
       <c r="AW11" s="23"/>
       <c r="AX11" s="23" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="AY11" s="23" t="s">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="AZ11" s="23" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="BA11" s="23" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="BB11" s="23" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="BC11" s="23" t="s">
         <v>89</v>
@@ -2953,10 +2867,10 @@
     </row>
     <row r="12" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="23" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="D12" s="23" t="s">
         <v>83</v>
@@ -2971,10 +2885,10 @@
         <v>86</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="J12" s="23" t="s">
         <v>89</v>
@@ -2992,10 +2906,10 @@
         <v>91</v>
       </c>
       <c r="O12" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="P12" s="23" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="Q12" s="24" t="n">
         <v>0.18</v>
@@ -3013,13 +2927,13 @@
       </c>
       <c r="V12" s="23"/>
       <c r="W12" s="23" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="X12" s="23" t="s">
         <v>95</v>
       </c>
       <c r="Y12" s="23" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="Z12" s="23" t="n">
         <v>1</v>
@@ -3037,7 +2951,7 @@
         <v>99</v>
       </c>
       <c r="AE12" s="23" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="AF12" s="23" t="s">
         <v>89</v>
@@ -3065,7 +2979,7 @@
       </c>
       <c r="AN12" s="23"/>
       <c r="AO12" s="23" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="AP12" s="23" t="s">
         <v>104</v>
@@ -3077,30 +2991,26 @@
         <v>102</v>
       </c>
       <c r="AS12" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="AT12" s="27" t="s">
-        <v>223</v>
-      </c>
-      <c r="AU12" s="27" t="s">
-        <v>224</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="AT12" s="23"/>
+      <c r="AU12" s="23"/>
       <c r="AV12" s="23"/>
       <c r="AW12" s="23"/>
       <c r="AX12" s="23" t="s">
-        <v>225</v>
+        <v>207</v>
       </c>
       <c r="AY12" s="23" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="AZ12" s="23" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="BA12" s="23" t="s">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="BB12" s="23" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="BC12" s="23" t="s">
         <v>89</v>
@@ -3118,33 +3028,15 @@
     <mergeCell ref="AX1:BD1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="AS4" r:id="rId1" display="https://drive.google.com/file/d/1ojWdYnCJPWy2Xry-GwUgrazq6poDKA46/view?usp=sharing"/>
-    <hyperlink ref="AT4" r:id="rId2" display="https://drive.google.com/file/d/1MDYo51NrfGPkuBgTsGfLFFiV2VMNFJL-/view?usp=sharing"/>
-    <hyperlink ref="AU4" r:id="rId3" display="https://drive.google.com/file/d/1S0NjAbs1t2PnUT5WwkgoCC0DZEd7LZkj/view?usp=sharing"/>
-    <hyperlink ref="AS5" r:id="rId4" display="https://drive.google.com/file/d/1hjMuxQFD3OMfm1LAD-V9o5ORxUsBJaf3/view?usp=sharing"/>
-    <hyperlink ref="AT5" r:id="rId5" display="https://drive.google.com/file/d/1TnwNh-Ns5sfxEvVs9yuNhuzc81QPA1w5/view?usp=sharing"/>
-    <hyperlink ref="AU5" r:id="rId6" display="https://drive.google.com/file/d/1yuGNdOGkSV1Ue9oAf1j-b1rGPck6FXjM/view?usp=sharing"/>
-    <hyperlink ref="AS6" r:id="rId7" display="https://drive.google.com/file/d/1UdZHk7EgjZvW_xLjQIhK8M6aPiFte948/view?usp=sharing"/>
-    <hyperlink ref="AT6" r:id="rId8" display="https://drive.google.com/file/d/14hvZZGQhXwXwRrOJJdKCLJE3medAwp9Q/view?usp=sharing"/>
-    <hyperlink ref="AU6" r:id="rId9" display="https://drive.google.com/file/d/10rPjU5WyUX4xxGCrZ5h_yqB_zt8JCHxS/view?usp=sharing"/>
-    <hyperlink ref="AS7" r:id="rId10" display="https://drive.google.com/file/d/1umHrvjv06YnpqEHCoWrbCxMw4MTp6JzN/view?usp=sharing"/>
-    <hyperlink ref="AT7" r:id="rId11" display="https://drive.google.com/file/d/1i1mF2QO-_Vq26uORz9_jA3_I2tlEKnhk/view?usp=sharing"/>
-    <hyperlink ref="AU7" r:id="rId12" display="https://drive.google.com/file/d/1NH_1N1TkxW9ACirUh1FoaU31rp2DxRXN/view?usp=sharing"/>
-    <hyperlink ref="AS8" r:id="rId13" display="https://drive.google.com/file/d/1zAMS6K6sWCh_NqpWCm7SdjZNAMQ2uKtR/view?usp=sharing"/>
-    <hyperlink ref="AT8" r:id="rId14" display="https://drive.google.com/file/d/1fmFzwud8FrECv-RwU9OfIZuVjcbvNmmj/view?usp=sharing"/>
-    <hyperlink ref="AU8" r:id="rId15" display="https://drive.google.com/file/d/1FR3-uayY0T8GsnBWnZIYNRBbWr2clFur/view?usp=sharing"/>
-    <hyperlink ref="AS9" r:id="rId16" display="https://drive.google.com/file/d/1cTQRotWPDhHA_RtCwpVskOSR-sMYpr8K/view?usp=sharing"/>
-    <hyperlink ref="AT9" r:id="rId17" display="https://drive.google.com/file/d/1rXHQPKDfXCNRms8f1pN1lp0gGPi8A_-f/view?usp=sharing"/>
-    <hyperlink ref="AU9" r:id="rId18" display="https://drive.google.com/file/d/16YmfYP-0aJSy9OVJtyX-LoFR-6UuPD_y/view?usp=sharing"/>
-    <hyperlink ref="AS10" r:id="rId19" display="https://drive.google.com/file/d/18wk--a6LK37uWyiUke-j8VBr8GPyXe9p/view?usp=sharing"/>
-    <hyperlink ref="AT10" r:id="rId20" display="https://drive.google.com/file/d/1TYR8F2kH5989Ig2XyV-VJV7UWFag3b4W/view?usp=sharing"/>
-    <hyperlink ref="AU10" r:id="rId21" display="https://drive.google.com/file/d/1We8eX5a5-Ookx9D6GWYnZqb3-GDq9oTQ/view?usp=sharing"/>
-    <hyperlink ref="AS11" r:id="rId22" display="https://drive.google.com/file/d/1hUNAArHtCA4s-z369ryqC0Vus224hnjC/view?usp=sharing"/>
-    <hyperlink ref="AT11" r:id="rId23" display="https://drive.google.com/file/d/1MbocXL41HpC-Y-OXbX9pw4Odbk34tyIb/view?usp=sharing"/>
-    <hyperlink ref="AU11" r:id="rId24" display="https://drive.google.com/file/d/1hIKX0vLKsZw5VYjm_Eq6gKU38G4PwXq7/view?usp=sharing"/>
-    <hyperlink ref="AS12" r:id="rId25" display="https://drive.google.com/file/d/14xwU3kZ_G1qqrzXsCocsRew3Pr2ogTmE/view?usp=sharing"/>
-    <hyperlink ref="AT12" r:id="rId26" display="https://drive.google.com/file/d/1hOabuPnhlME44_vUeBXzDIjcRipyS1b0/view?usp=sharing"/>
-    <hyperlink ref="AU12" r:id="rId27" display="https://drive.google.com/file/d/11kC1g7ONIDJLAFmnj-hIU9_AMVgZJJq_/view?usp=sharing"/>
+    <hyperlink ref="AS4" r:id="rId1" display="https://drive.google.com/drive/folders/1yP0mxPJhdgPbR_s79_MmLFm8sYI0-gdb?usp=sharing"/>
+    <hyperlink ref="AS5" r:id="rId2" display="https://drive.google.com/drive/folders/1jFOX8x5PyO-MDKmMh9RHKWpgABZ-T2jI?usp=sharing"/>
+    <hyperlink ref="AS6" r:id="rId3" display="https://drive.google.com/drive/folders/1AXhoTNn1WFYVBmDmYVGPnRJLoNuc1GcK?usp=sharing"/>
+    <hyperlink ref="AS7" r:id="rId4" display="https://drive.google.com/drive/folders/1Kn3zQ2TjI-Z_pSl68ySUC-9QEAPxW7MU?usp=sharing"/>
+    <hyperlink ref="AS8" r:id="rId5" display="https://drive.google.com/drive/folders/1--OQ7u1bta3auUdssAOvANlM_OuQiwSh?usp=sharing"/>
+    <hyperlink ref="AS9" r:id="rId6" display="https://drive.google.com/drive/folders/1c0mnshaI1ujk8pprI4qJ7qiXcjMrVSHs?usp=sharing"/>
+    <hyperlink ref="AS10" r:id="rId7" display="https://drive.google.com/drive/folders/1W2AU9JUfyl_QFj6OUIehl_ix4VNvqI-W?usp=sharing"/>
+    <hyperlink ref="AS11" r:id="rId8" display="https://drive.google.com/drive/folders/1k3T5Ys14H5-t8kIDUY1nKzM9oEpxfpYV?usp=sharing"/>
+    <hyperlink ref="AS12" r:id="rId9" display="https://drive.google.com/drive/folders/1EFJ1SJS3AjAbHOzTtWMO0-ieMek5WyxN?usp=sharing"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>